<commit_message>
Revision update: 1.5x data, fixed test set, stratified model selection
- Rate tables at the 1.5x hydrolysis control, labelled from the scope workbook
  (scripts/build_rate_tables.py); 4-fluorobenzoyl chloride batches 1A/2B/3C
  combined by geometric mean (PRISM_rates_all.xlsx keeps every value).
- Fixed held-out test set: acyl chlorides 2, 18, 25; amines 18, 21, 23.
- Descriptor set and learner selected by repeated class-stratified validation
  inside the training pool (20 draws): Tier 2 (reduced) + LightGBM.
- Held-out test accuracy 0.83, rate R2 0.79; excluded scope 0.87; drug scope
  7/11; all three pooled 0.83.
- Data summary analysis; data dictionary; README and docs/RESULTS.md updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JkLzRCnHQm67YFeR7F5Ysw
</commit_message>
<xml_diff>
--- a/analysis/data/PRISM_vs_hammett.xlsx
+++ b/analysis/data/PRISM_vs_hammett.xlsx
@@ -573,7 +573,7 @@
         <v>82.6823</v>
       </c>
       <c r="H2" t="n">
-        <v>98.4615384615384</v>
+        <v>144.9314603705081</v>
       </c>
       <c r="I2" t="n">
         <v>22.3</v>
@@ -607,7 +607,7 @@
         <v>1.129406892</v>
       </c>
       <c r="T2" t="n">
-        <v>1.189252705113653</v>
+        <v>1.357148756075249</v>
       </c>
       <c r="U2" t="n">
         <v>-1.5</v>
@@ -656,7 +656,7 @@
         <v>29.6559</v>
       </c>
       <c r="H3" t="n">
-        <v>21.3817669393666</v>
+        <v>26.73704928902369</v>
       </c>
       <c r="I3" t="n">
         <v>22.7</v>
@@ -690,7 +690,7 @@
         <v>0.6841054519999999</v>
       </c>
       <c r="T3" t="n">
-        <v>0.5260296792117499</v>
+        <v>0.6230995644381428</v>
       </c>
       <c r="U3" t="n">
         <v>-1.1</v>
@@ -739,7 +739,7 @@
         <v>19.0456</v>
       </c>
       <c r="H4" t="n">
-        <v>20.6207473711021</v>
+        <v>31.0665463857562</v>
       </c>
       <c r="I4" t="n">
         <v>22.7</v>
@@ -773,7 +773,7 @@
         <v>0.491789002</v>
       </c>
       <c r="T4" t="n">
-        <v>0.5102904894215514</v>
+        <v>0.6882790639443815</v>
       </c>
       <c r="U4" t="n">
         <v>-1.1</v>
@@ -948,7 +948,7 @@
         <v>6.1377</v>
       </c>
       <c r="H7" t="n">
-        <v>6.36815920398009</v>
+        <v>6.368159203980089</v>
       </c>
       <c r="I7" t="n">
         <v>23.8</v>
@@ -1496,9 +1496,7 @@
       <c r="G14" t="n">
         <v>3.6466</v>
       </c>
-      <c r="H14" t="n">
-        <v>7.35632183908046</v>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
         <v>22.6</v>
       </c>
@@ -1530,9 +1528,7 @@
       <c r="S14" t="n">
         <v>-0.273650256</v>
       </c>
-      <c r="T14" t="n">
-        <v>0.051706823073877</v>
-      </c>
+      <c r="T14" t="inlineStr"/>
       <c r="U14" t="n">
         <v>1.7</v>
       </c>
@@ -1545,11 +1541,7 @@
       <c r="X14" t="n">
         <v>-0.146609175</v>
       </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>low_confidence_order_of_magnitude</t>
-        </is>
-      </c>
+      <c r="Y14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1847,7 +1839,7 @@
         <v>0.354403676</v>
       </c>
       <c r="T18" t="n">
-        <v>0.2588323158695251</v>
+        <v>0.2588323158695252</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>
@@ -1896,7 +1888,7 @@
         <v>12.9576</v>
       </c>
       <c r="H19" t="n">
-        <v>21.0526315789473</v>
+        <v>20.9749171793658</v>
       </c>
       <c r="I19" t="n">
         <v>20.3</v>
@@ -1930,7 +1922,7 @@
         <v>0.276986186</v>
       </c>
       <c r="T19" t="n">
-        <v>0.5083524920837403</v>
+        <v>0.5067463563766677</v>
       </c>
       <c r="U19" t="n">
         <v>-0.6</v>
@@ -1946,7 +1938,7 @@
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>high_confidence</t>
+          <t>medium_confidence</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2005,7 @@
         <v>0.293180672</v>
       </c>
       <c r="T20" t="n">
-        <v>0.4076563940873822</v>
+        <v>0.4076563940873821</v>
       </c>
       <c r="U20" t="n">
         <v>0.7</v>
@@ -2062,7 +2054,7 @@
         <v>18.9571</v>
       </c>
       <c r="H21" t="n">
-        <v>30.616958099637</v>
+        <v>30.61695809963701</v>
       </c>
       <c r="I21" t="n">
         <v>20.4</v>
@@ -2096,7 +2088,7 @@
         <v>0.442233518</v>
       </c>
       <c r="T21" t="n">
-        <v>0.6710081415598469</v>
+        <v>0.671008141559847</v>
       </c>
       <c r="U21" t="n">
         <v>-0.5</v>
@@ -2145,7 +2137,7 @@
         <v>24.5018</v>
       </c>
       <c r="H22" t="n">
-        <v>71.111111111111</v>
+        <v>71.11111111111099</v>
       </c>
       <c r="I22" t="n">
         <v>20.3</v>
@@ -2228,7 +2220,7 @@
         <v>113.83</v>
       </c>
       <c r="H23" t="n">
-        <v>120</v>
+        <v>159.9999999999999</v>
       </c>
       <c r="I23" t="n">
         <v>19.7</v>
@@ -2262,7 +2254,7 @@
         <v>1.220718353</v>
       </c>
       <c r="T23" t="n">
-        <v>1.264227347756233</v>
+        <v>1.389166084364533</v>
       </c>
       <c r="U23" t="n">
         <v>-1.2</v>
@@ -2278,7 +2270,7 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>medium_confidence</t>
+          <t>low_confidence_order_of_magnitude</t>
         </is>
       </c>
     </row>

</xml_diff>